<commit_message>
Ingreso de producto MTS-0063: Disco Solido SSD 2.5 SATA 240GB ADATA SU650 y sincronizacion a catalogo web
</commit_message>
<xml_diff>
--- a/inventario_max_technology_store.xlsx
+++ b/inventario_max_technology_store.xlsx
@@ -7571,7 +7571,119 @@
         </is>
       </c>
     </row>
-    <row r="66"/>
+    <row r="66">
+      <c r="A66" s="77" t="inlineStr">
+        <is>
+          <t>MTS-0063</t>
+        </is>
+      </c>
+      <c r="B66" s="67" t="inlineStr">
+        <is>
+          <t>Disco Estado Sólido SSD 2.5" SATA III 240GB ADATA Ultimate SU650</t>
+        </is>
+      </c>
+      <c r="C66" s="68" t="inlineStr">
+        <is>
+          <t>Almacenamiento y Memorias</t>
+        </is>
+      </c>
+      <c r="D66" s="68" t="inlineStr">
+        <is>
+          <t>ADATA</t>
+        </is>
+      </c>
+      <c r="E66" s="69" t="inlineStr">
+        <is>
+          <t>ASU650SS-240GT-R</t>
+        </is>
+      </c>
+      <c r="F66" s="69" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="G66" s="69" t="inlineStr">
+        <is>
+          <t>4713435793672</t>
+        </is>
+      </c>
+      <c r="H66" s="69" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="I66" s="70" t="inlineStr">
+        <is>
+          <t>🟢 En Stock</t>
+        </is>
+      </c>
+      <c r="J66" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="K66" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="L66" s="69" t="inlineStr">
+        <is>
+          <t>Vitrina Accesorios / Taller</t>
+        </is>
+      </c>
+      <c r="M66" s="78" t="n">
+        <v>169000</v>
+      </c>
+      <c r="N66" s="79" t="n">
+        <v>0.295833</v>
+      </c>
+      <c r="O66" s="80">
+        <f>IF(N66&lt;1, ROUNDUP(M66/(1-N66), -3), M66)</f>
+        <v/>
+      </c>
+      <c r="P66" s="79" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="Q66" s="78">
+        <f>IF((1-N66-P66)&gt;0, ROUNDUP((M66+IF(O66&gt;=90000,20000,0))/(1-N66-P66), -3), O66)</f>
+        <v/>
+      </c>
+      <c r="R66" s="78">
+        <f>O66</f>
+        <v/>
+      </c>
+      <c r="S66" s="78">
+        <f>O66-M66</f>
+        <v/>
+      </c>
+      <c r="T66" s="79">
+        <f>IF(O66&gt;0, (O66-M66)/O66, 0)</f>
+        <v/>
+      </c>
+      <c r="U66" s="69" t="inlineStr">
+        <is>
+          <t>36 Meses (3 Años ADATA)</t>
+        </is>
+      </c>
+      <c r="V66" s="68" t="inlineStr">
+        <is>
+          <t>IMAGENES DE PRODUCTOS/adata 240 gb sata.jpg</t>
+        </is>
+      </c>
+      <c r="W66" s="68" t="inlineStr">
+        <is>
+          <t>• Capacidad: 240 GB
+• Factor de forma: 2.5 pulgadas (7 mm de grosor)
+• Interfaz: SATA III 6Gb/s (retrocompatible con SATA II)
+• Velocidad de lectura secuencial: Hasta 520 MB/s
+• Velocidad de escritura secuencial: Hasta 450 MB/s
+• Tecnología: Memoria 3D NAND Flash con caché SLC y corrección de errores ECC
+• Compatibilidad: Ideal para actualizar computadores de escritorio o portátiles y multiplicar su velocidad.</t>
+        </is>
+      </c>
+      <c r="X66" s="68" t="inlineStr">
+        <is>
+          <t>Producto nuevo remisionado. Referencia SU650.</t>
+        </is>
+      </c>
+    </row>
     <row r="67"/>
     <row r="68"/>
     <row r="69"/>

</xml_diff>

<commit_message>
Ingreso de productos MTS-0064 (Caja Externa HDD/SSD POSUGEAR) y MTS-0065 (Bateria UPS Powest 12V 7.5Ah 2u) con sincronizacion a Excel y GitHub Pages
</commit_message>
<xml_diff>
--- a/inventario_max_technology_store.xlsx
+++ b/inventario_max_technology_store.xlsx
@@ -7684,8 +7684,228 @@
         </is>
       </c>
     </row>
-    <row r="67"/>
-    <row r="68"/>
+    <row r="67">
+      <c r="A67" s="77" t="inlineStr">
+        <is>
+          <t>MTS-0064</t>
+        </is>
+      </c>
+      <c r="B67" s="67" t="inlineStr">
+        <is>
+          <t>Caja / Cofre Externo para Disco Duro 2.5" SATA a USB 3.0 Transparente POSUGEAR</t>
+        </is>
+      </c>
+      <c r="C67" s="68" t="inlineStr">
+        <is>
+          <t>Almacenamiento y Memorias</t>
+        </is>
+      </c>
+      <c r="D67" s="68" t="inlineStr">
+        <is>
+          <t>POSUGEAR</t>
+        </is>
+      </c>
+      <c r="E67" s="69" t="inlineStr">
+        <is>
+          <t>B0C9TGQ8F5</t>
+        </is>
+      </c>
+      <c r="F67" s="69" t="inlineStr">
+        <is>
+          <t>Transparente</t>
+        </is>
+      </c>
+      <c r="G67" s="69" t="inlineStr">
+        <is>
+          <t>Sin código</t>
+        </is>
+      </c>
+      <c r="H67" s="69" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="I67" s="70" t="inlineStr">
+        <is>
+          <t>🟢 En Stock</t>
+        </is>
+      </c>
+      <c r="J67" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="K67" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="L67" s="69" t="inlineStr">
+        <is>
+          <t>Vitrina Accesorios / Taller</t>
+        </is>
+      </c>
+      <c r="M67" s="78" t="n">
+        <v>21700</v>
+      </c>
+      <c r="N67" s="79" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="O67" s="80">
+        <f>IF(N67&lt;1, ROUNDUP(M67/(1-N67), -3), M67)</f>
+        <v/>
+      </c>
+      <c r="P67" s="79" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="Q67" s="78">
+        <f>IF((1-N67-P67)&gt;0, ROUNDUP((M67+IF(O67&gt;=90000,20000,0))/(1-N67-P67), -3), O67)</f>
+        <v/>
+      </c>
+      <c r="R67" s="78">
+        <f>O67</f>
+        <v/>
+      </c>
+      <c r="S67" s="78">
+        <f>O67-M67</f>
+        <v/>
+      </c>
+      <c r="T67" s="79">
+        <f>IF(O67&gt;0, (O67-M67)/O67, 0)</f>
+        <v/>
+      </c>
+      <c r="U67" s="69" t="inlineStr">
+        <is>
+          <t>6 Meses</t>
+        </is>
+      </c>
+      <c r="V67" s="68" t="inlineStr">
+        <is>
+          <t>IMAGENES DE PRODUCTOS/61YDB9nALmL._AC_SL1500_.jpg</t>
+        </is>
+      </c>
+      <c r="W67" s="68" t="inlineStr">
+        <is>
+          <t>• Compatibilidad: Discos duros (HDD) y unidades de estado sólido (SSD) de 2.5" SATA I/II/III (7mm a 9.5mm, hasta 6 TB)
+• Conexión: Interfaz USB 3.0 con soporte UASP de alta velocidad (transferencias de hasta 5 Gbps)
+• Diseño: Carcasa transparente en policarbonato ultrarresistente (permite ver qué disco está instalado)
+• Instalación: 100% libre de herramientas (Tool-Free), apertura fácil mediante tapa deslizable
+• Plug &amp; Play: Conexión directa sin drivers en Windows, macOS, Linux, Smart TV, PS4, PS5 y Xbox.</t>
+        </is>
+      </c>
+      <c r="X67" s="68" t="inlineStr">
+        <is>
+          <t>Carcasa transparente para disco duro externo 2.5 SATA. Pedido Amazon 111-4517322-7785837.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="77" t="inlineStr">
+        <is>
+          <t>MTS-0065</t>
+        </is>
+      </c>
+      <c r="B68" s="67" t="inlineStr">
+        <is>
+          <t>Batería Seca Recargable para UPS 12V 7.5Ah Powest (FL1275GS)</t>
+        </is>
+      </c>
+      <c r="C68" s="68" t="inlineStr">
+        <is>
+          <t>Energía y Respaldo / UPS</t>
+        </is>
+      </c>
+      <c r="D68" s="68" t="inlineStr">
+        <is>
+          <t>Powest</t>
+        </is>
+      </c>
+      <c r="E68" s="69" t="inlineStr">
+        <is>
+          <t>FL1275GS</t>
+        </is>
+      </c>
+      <c r="F68" s="69" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="G68" s="69" t="inlineStr">
+        <is>
+          <t>Sin código</t>
+        </is>
+      </c>
+      <c r="H68" s="69" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="I68" s="70" t="inlineStr">
+        <is>
+          <t>🟢 En Stock</t>
+        </is>
+      </c>
+      <c r="J68" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="K68" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="L68" s="69" t="inlineStr">
+        <is>
+          <t>Estante Baterías / Taller</t>
+        </is>
+      </c>
+      <c r="M68" s="78" t="n">
+        <v>45000</v>
+      </c>
+      <c r="N68" s="79" t="n">
+        <v>0.307692</v>
+      </c>
+      <c r="O68" s="80">
+        <f>IF(N68&lt;1, ROUNDUP(M68/(1-N68), -3), M68)</f>
+        <v/>
+      </c>
+      <c r="P68" s="79" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="Q68" s="78">
+        <f>IF((1-N68-P68)&gt;0, ROUNDUP((M68+IF(O68&gt;=90000,20000,0))/(1-N68-P68), -3), O68)</f>
+        <v/>
+      </c>
+      <c r="R68" s="78">
+        <f>O68</f>
+        <v/>
+      </c>
+      <c r="S68" s="78">
+        <f>O68-M68</f>
+        <v/>
+      </c>
+      <c r="T68" s="79">
+        <f>IF(O68&gt;0, (O68-M68)/O68, 0)</f>
+        <v/>
+      </c>
+      <c r="U68" s="69" t="inlineStr">
+        <is>
+          <t>12 Meses (1 Año Powest)</t>
+        </is>
+      </c>
+      <c r="V68" s="68" t="inlineStr">
+        <is>
+          <t>IMAGENES DE PRODUCTOS/bateria ups powest 12v7ah.jpg</t>
+        </is>
+      </c>
+      <c r="W68" s="68" t="inlineStr">
+        <is>
+          <t>• Voltaje nominal: 12V DC
+• Capacidad: 7.5 Ah / 20Hr
+• Tecnología: VRLA / AGM (Plomo-Ácido sellada libre de mantenimiento, a prueba de fugas)
+• Terminales: Tipo F1 / Faston 187 (estándar para fácil conexión)
+• Aplicaciones: Reemplazo ideal para UPS interactivas (APC, Unitec, CDP, Powest, Forza), sistemas de alarma, cercas eléctricas, iluminación y plantas solares.</t>
+        </is>
+      </c>
+      <c r="X68" s="68" t="inlineStr">
+        <is>
+          <t>2 unidades físicas nuevas en taller. Modelo FL1275GS.</t>
+        </is>
+      </c>
+    </row>
     <row r="69"/>
     <row r="70"/>
     <row r="71"/>

</xml_diff>

<commit_message>
Ingreso de lote de productos MTS-0066 a MTS-0071 (Camaras IMOU y Dahua, MicroSD Sandisk 128GB, Diadema Genius, Cable Serial Jaltech y Ventilador 4010) y blindaje de formulas comerciales en Excel y catalogo web
</commit_message>
<xml_diff>
--- a/inventario_max_technology_store.xlsx
+++ b/inventario_max_technology_store.xlsx
@@ -1256,7 +1256,7 @@
         <v>580115</v>
       </c>
       <c r="N4" s="76" t="n">
-        <v>0.3</v>
+        <v>0.3002223163115999</v>
       </c>
       <c r="O4" s="77">
         <f>IF(N4&lt;1, ROUNDUP(M4/(1-N4), -3), M4)</f>
@@ -1359,7 +1359,7 @@
         <v>131293</v>
       </c>
       <c r="N5" s="76" t="n">
-        <v>0.2</v>
+        <v>0.2042800259395512</v>
       </c>
       <c r="O5" s="77">
         <f>IF(N5&lt;1, ROUNDUP(M5/(1-N5), -3), M5)</f>
@@ -1462,7 +1462,7 @@
         <v>39705</v>
       </c>
       <c r="N6" s="76" t="n">
-        <v>0.11</v>
+        <v>0.1176470588235294</v>
       </c>
       <c r="O6" s="77">
         <f>IF(N6&lt;1, ROUNDUP(M6/(1-N6), -3), M6)</f>
@@ -1565,7 +1565,7 @@
         <v>90586</v>
       </c>
       <c r="N7" s="76" t="n">
-        <v>0.21</v>
+        <v>0.2122888025113262</v>
       </c>
       <c r="O7" s="77">
         <f>IF(N7&lt;1, ROUNDUP(M7/(1-N7), -3), M7)</f>
@@ -1668,7 +1668,7 @@
         <v>59921</v>
       </c>
       <c r="N8" s="76" t="n">
-        <v>0.14</v>
+        <v>0.1439734853355048</v>
       </c>
       <c r="O8" s="77">
         <f>IF(N8&lt;1, ROUNDUP(M8/(1-N8), -3), M8)</f>
@@ -1771,7 +1771,7 @@
         <v>43435</v>
       </c>
       <c r="N9" s="76" t="n">
-        <v>0.2</v>
+        <v>0.2102583683339697</v>
       </c>
       <c r="O9" s="77">
         <f>IF(N9&lt;1, ROUNDUP(M9/(1-N9), -3), M9)</f>
@@ -1874,7 +1874,7 @@
         <v>16180</v>
       </c>
       <c r="N10" s="76" t="n">
-        <v>0.35</v>
+        <v>0.3527741109644386</v>
       </c>
       <c r="O10" s="77">
         <f>IF(N10&lt;1, ROUNDUP(M10/(1-N10), -3), M10)</f>
@@ -1977,7 +1977,7 @@
         <v>45000</v>
       </c>
       <c r="N11" s="76" t="n">
-        <v>0.25</v>
+        <v>0.2499874997916632</v>
       </c>
       <c r="O11" s="77">
         <f>IF(N11&lt;1, ROUNDUP(M11/(1-N11), -3), M11)</f>
@@ -2080,7 +2080,7 @@
         <v>10948</v>
       </c>
       <c r="N12" s="76" t="n">
-        <v>0.25</v>
+        <v>0.2700846723114875</v>
       </c>
       <c r="O12" s="77">
         <f>IF(N12&lt;1, ROUNDUP(M12/(1-N12), -3), M12)</f>
@@ -2179,7 +2179,7 @@
         <v>10000</v>
       </c>
       <c r="N13" s="76" t="n">
-        <v>0.3</v>
+        <v>0.3332888859257284</v>
       </c>
       <c r="O13" s="77">
         <f>IF(N13&lt;1, ROUNDUP(M13/(1-N13), -3), M13)</f>
@@ -2282,7 +2282,7 @@
         <v>25000</v>
       </c>
       <c r="N14" s="76" t="n">
-        <v>0.44</v>
+        <v>0.4444320984910776</v>
       </c>
       <c r="O14" s="77">
         <f>IF(N14&lt;1, ROUNDUP(M14/(1-N14), -3), M14)</f>
@@ -2389,7 +2389,7 @@
         <v>30000</v>
       </c>
       <c r="N15" s="76" t="n">
-        <v>0.4</v>
+        <v>0.3999879997599952</v>
       </c>
       <c r="O15" s="77">
         <f>IF(N15&lt;1, ROUNDUP(M15/(1-N15), -3), M15)</f>
@@ -2496,7 +2496,7 @@
         <v>30000</v>
       </c>
       <c r="N16" s="76" t="n">
-        <v>0.4</v>
+        <v>0.3999879997599952</v>
       </c>
       <c r="O16" s="77">
         <f>IF(N16&lt;1, ROUNDUP(M16/(1-N16), -3), M16)</f>
@@ -2603,7 +2603,7 @@
         <v>30000</v>
       </c>
       <c r="N17" s="76" t="n">
-        <v>0.4</v>
+        <v>0.3999879997599952</v>
       </c>
       <c r="O17" s="77">
         <f>IF(N17&lt;1, ROUNDUP(M17/(1-N17), -3), M17)</f>
@@ -2710,7 +2710,7 @@
         <v>20000</v>
       </c>
       <c r="N18" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O18" s="77">
         <f>IF(N18&lt;1, ROUNDUP(M18/(1-N18), -3), M18)</f>
@@ -2817,7 +2817,7 @@
         <v>20000</v>
       </c>
       <c r="N19" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O19" s="77">
         <f>IF(N19&lt;1, ROUNDUP(M19/(1-N19), -3), M19)</f>
@@ -2924,7 +2924,7 @@
         <v>20000</v>
       </c>
       <c r="N20" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O20" s="77">
         <f>IF(N20&lt;1, ROUNDUP(M20/(1-N20), -3), M20)</f>
@@ -3031,7 +3031,7 @@
         <v>20000</v>
       </c>
       <c r="N21" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O21" s="77">
         <f>IF(N21&lt;1, ROUNDUP(M21/(1-N21), -3), M21)</f>
@@ -3138,7 +3138,7 @@
         <v>20000</v>
       </c>
       <c r="N22" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O22" s="77">
         <f>IF(N22&lt;1, ROUNDUP(M22/(1-N22), -3), M22)</f>
@@ -3245,7 +3245,7 @@
         <v>20000</v>
       </c>
       <c r="N23" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O23" s="77">
         <f>IF(N23&lt;1, ROUNDUP(M23/(1-N23), -3), M23)</f>
@@ -3352,7 +3352,7 @@
         <v>20000</v>
       </c>
       <c r="N24" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O24" s="77">
         <f>IF(N24&lt;1, ROUNDUP(M24/(1-N24), -3), M24)</f>
@@ -3459,7 +3459,7 @@
         <v>20000</v>
       </c>
       <c r="N25" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O25" s="77">
         <f>IF(N25&lt;1, ROUNDUP(M25/(1-N25), -3), M25)</f>
@@ -3566,7 +3566,7 @@
         <v>20000</v>
       </c>
       <c r="N26" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O26" s="77">
         <f>IF(N26&lt;1, ROUNDUP(M26/(1-N26), -3), M26)</f>
@@ -3673,7 +3673,7 @@
         <v>20000</v>
       </c>
       <c r="N27" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O27" s="77">
         <f>IF(N27&lt;1, ROUNDUP(M27/(1-N27), -3), M27)</f>
@@ -3780,7 +3780,7 @@
         <v>20000</v>
       </c>
       <c r="N28" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O28" s="77">
         <f>IF(N28&lt;1, ROUNDUP(M28/(1-N28), -3), M28)</f>
@@ -3887,7 +3887,7 @@
         <v>20000</v>
       </c>
       <c r="N29" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O29" s="77">
         <f>IF(N29&lt;1, ROUNDUP(M29/(1-N29), -3), M29)</f>
@@ -3994,7 +3994,7 @@
         <v>20000</v>
       </c>
       <c r="N30" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O30" s="77">
         <f>IF(N30&lt;1, ROUNDUP(M30/(1-N30), -3), M30)</f>
@@ -4101,7 +4101,7 @@
         <v>20000</v>
       </c>
       <c r="N31" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O31" s="77">
         <f>IF(N31&lt;1, ROUNDUP(M31/(1-N31), -3), M31)</f>
@@ -4208,7 +4208,7 @@
         <v>20000</v>
       </c>
       <c r="N32" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O32" s="77">
         <f>IF(N32&lt;1, ROUNDUP(M32/(1-N32), -3), M32)</f>
@@ -4315,7 +4315,7 @@
         <v>20000</v>
       </c>
       <c r="N33" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O33" s="77">
         <f>IF(N33&lt;1, ROUNDUP(M33/(1-N33), -3), M33)</f>
@@ -4422,7 +4422,7 @@
         <v>20000</v>
       </c>
       <c r="N34" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O34" s="77">
         <f>IF(N34&lt;1, ROUNDUP(M34/(1-N34), -3), M34)</f>
@@ -4529,7 +4529,7 @@
         <v>20000</v>
       </c>
       <c r="N35" s="76" t="n">
-        <v>0.33</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O35" s="77">
         <f>IF(N35&lt;1, ROUNDUP(M35/(1-N35), -3), M35)</f>
@@ -4632,7 +4632,7 @@
         <v>158550</v>
       </c>
       <c r="N36" s="76" t="n">
-        <v>0.28</v>
+        <v>0.2825759392576437</v>
       </c>
       <c r="O36" s="77">
         <f>IF(N36&lt;1, ROUNDUP(M36/(1-N36), -3), M36)</f>
@@ -4735,7 +4735,7 @@
         <v>432546</v>
       </c>
       <c r="N37" s="76" t="n">
-        <v>0.25</v>
+        <v>0.2503522536434205</v>
       </c>
       <c r="O37" s="77">
         <f>IF(N37&lt;1, ROUNDUP(M37/(1-N37), -3), M37)</f>
@@ -4838,7 +4838,7 @@
         <v>163096</v>
       </c>
       <c r="N38" s="76" t="n">
-        <v>0.3</v>
+        <v>0.3000141631509148</v>
       </c>
       <c r="O38" s="77">
         <f>IF(N38&lt;1, ROUNDUP(M38/(1-N38), -3), M38)</f>
@@ -4941,7 +4941,7 @@
         <v>265738</v>
       </c>
       <c r="N39" s="76" t="n">
-        <v>0.25</v>
+        <v>0.2514401449018167</v>
       </c>
       <c r="O39" s="77">
         <f>IF(N39&lt;1, ROUNDUP(M39/(1-N39), -3), M39)</f>
@@ -5048,7 +5048,7 @@
         <v>311071</v>
       </c>
       <c r="N40" s="76" t="n">
-        <v>0.20238</v>
+        <v>0.2023800061025798</v>
       </c>
       <c r="O40" s="77">
         <f>IF(N40&lt;1, ROUNDUP(M40/(1-N40), -3), M40)</f>
@@ -5157,7 +5157,7 @@
         <v>310243</v>
       </c>
       <c r="N41" s="76" t="n">
-        <v>0.25</v>
+        <v>0.2506189628477363</v>
       </c>
       <c r="O41" s="77">
         <f>IF(N41&lt;1, ROUNDUP(M41/(1-N41), -3), M41)</f>
@@ -5260,7 +5260,7 @@
         <v>2065526</v>
       </c>
       <c r="N42" s="76" t="n">
-        <v>0.18</v>
+        <v>0.1800211115605842</v>
       </c>
       <c r="O42" s="77">
         <f>IF(N42&lt;1, ROUNDUP(M42/(1-N42), -3), M42)</f>
@@ -5363,7 +5363,7 @@
         <v>2648576</v>
       </c>
       <c r="N43" s="76" t="n">
-        <v>0.16</v>
+        <v>0.1602483069905856</v>
       </c>
       <c r="O43" s="77">
         <f>IF(N43&lt;1, ROUNDUP(M43/(1-N43), -3), M43)</f>
@@ -5466,7 +5466,7 @@
         <v>2430833</v>
       </c>
       <c r="N44" s="76" t="n">
-        <v>0.18</v>
+        <v>0.1801572277090144</v>
       </c>
       <c r="O44" s="77">
         <f>IF(N44&lt;1, ROUNDUP(M44/(1-N44), -3), M44)</f>
@@ -5569,7 +5569,7 @@
         <v>8967320</v>
       </c>
       <c r="N45" s="76" t="n">
-        <v>0.15</v>
+        <v>0.1500169810442636</v>
       </c>
       <c r="O45" s="77">
         <f>IF(N45&lt;1, ROUNDUP(M45/(1-N45), -3), M45)</f>
@@ -5672,7 +5672,7 @@
         <v>142018</v>
       </c>
       <c r="N46" s="76" t="n">
-        <v>0.32</v>
+        <v>0.3204847870085503</v>
       </c>
       <c r="O46" s="77">
         <f>IF(N46&lt;1, ROUNDUP(M46/(1-N46), -3), M46)</f>
@@ -5775,7 +5775,7 @@
         <v>226100</v>
       </c>
       <c r="N47" s="76" t="n">
-        <v>0.3</v>
+        <v>0.2999978328106279</v>
       </c>
       <c r="O47" s="77">
         <f>IF(N47&lt;1, ROUNDUP(M47/(1-N47), -3), M47)</f>
@@ -5878,7 +5878,7 @@
         <v>87500</v>
       </c>
       <c r="N48" s="76" t="n">
-        <v>0.23</v>
+        <v>0.2324494074509426</v>
       </c>
       <c r="O48" s="77">
         <f>IF(N48&lt;1, ROUNDUP(M48/(1-N48), -3), M48)</f>
@@ -5977,7 +5977,7 @@
         <v>30244</v>
       </c>
       <c r="N49" s="76" t="n">
-        <v>0.39</v>
+        <v>0.3951079021580431</v>
       </c>
       <c r="O49" s="77">
         <f>IF(N49&lt;1, ROUNDUP(M49/(1-N49), -3), M49)</f>
@@ -6076,7 +6076,7 @@
         <v>154591</v>
       </c>
       <c r="N50" s="76" t="n">
-        <v>0.32</v>
+        <v>0.3219663244137035</v>
       </c>
       <c r="O50" s="77">
         <f>IF(N50&lt;1, ROUNDUP(M50/(1-N50), -3), M50)</f>
@@ -6179,7 +6179,7 @@
         <v>1393124</v>
       </c>
       <c r="N51" s="76" t="n">
-        <v>0.2</v>
+        <v>0.2002727900532664</v>
       </c>
       <c r="O51" s="77">
         <f>IF(N51&lt;1, ROUNDUP(M51/(1-N51), -3), M51)</f>
@@ -6282,7 +6282,7 @@
         <v>608875</v>
       </c>
       <c r="N52" s="76" t="n">
-        <v>0.25</v>
+        <v>0.2501530174298244</v>
       </c>
       <c r="O52" s="77">
         <f>IF(N52&lt;1, ROUNDUP(M52/(1-N52), -3), M52)</f>
@@ -6385,7 +6385,7 @@
         <v>29036</v>
       </c>
       <c r="N53" s="76" t="n">
-        <v>0.4</v>
+        <v>0.4074164778873038</v>
       </c>
       <c r="O53" s="77">
         <f>IF(N53&lt;1, ROUNDUP(M53/(1-N53), -3), M53)</f>
@@ -6488,7 +6488,7 @@
         <v>57126</v>
       </c>
       <c r="N54" s="76" t="n">
-        <v>0.38</v>
+        <v>0.3857353304874246</v>
       </c>
       <c r="O54" s="77">
         <f>IF(N54&lt;1, ROUNDUP(M54/(1-N54), -3), M54)</f>
@@ -6591,7 +6591,7 @@
         <v>95422</v>
       </c>
       <c r="N55" s="76" t="n">
-        <v>0.35</v>
+        <v>0.3508663324240301</v>
       </c>
       <c r="O55" s="77">
         <f>IF(N55&lt;1, ROUNDUP(M55/(1-N55), -3), M55)</f>
@@ -6694,7 +6694,7 @@
         <v>72202</v>
       </c>
       <c r="N56" s="76" t="n">
-        <v>0.38</v>
+        <v>0.3828836143898666</v>
       </c>
       <c r="O56" s="77">
         <f>IF(N56&lt;1, ROUNDUP(M56/(1-N56), -3), M56)</f>
@@ -6797,7 +6797,7 @@
         <v>253530</v>
       </c>
       <c r="N57" s="76" t="n">
-        <v>0.22</v>
+        <v>0.2222982279086746</v>
       </c>
       <c r="O57" s="77">
         <f>IF(N57&lt;1, ROUNDUP(M57/(1-N57), -3), M57)</f>
@@ -6900,7 +6900,7 @@
         <v>780250</v>
       </c>
       <c r="N58" s="76" t="n">
-        <v>0.25</v>
+        <v>0.2504795873963376</v>
       </c>
       <c r="O58" s="77">
         <f>IF(N58&lt;1, ROUNDUP(M58/(1-N58), -3), M58)</f>
@@ -7003,7 +7003,7 @@
         <v>39705</v>
       </c>
       <c r="N59" s="76" t="n">
-        <v>0.4</v>
+        <v>0.4073792146151435</v>
       </c>
       <c r="O59" s="77">
         <f>IF(N59&lt;1, ROUNDUP(M59/(1-N59), -3), M59)</f>
@@ -7110,7 +7110,7 @@
         <v>180000</v>
       </c>
       <c r="N60" s="76" t="n">
-        <v>0.2</v>
+        <v>0.199996444428642</v>
       </c>
       <c r="O60" s="77">
         <f>IF(N60&lt;1, ROUNDUP(M60/(1-N60), -3), M60)</f>
@@ -7219,7 +7219,7 @@
         <v>20000</v>
       </c>
       <c r="N61" s="86" t="n">
-        <v>0.32</v>
+        <v>0.3333111103703457</v>
       </c>
       <c r="O61" s="87">
         <f>IF(N61&lt;1, ROUNDUP(M61/(1-N61), -3), M61)</f>
@@ -7310,7 +7310,7 @@
         <v>8000</v>
       </c>
       <c r="N62" s="91" t="n">
-        <v>0.3</v>
+        <v>0.3332777731477623</v>
       </c>
       <c r="O62" s="92">
         <f>IF(N62&lt;1, ROUNDUP(M62/(1-N62), -3), M62)</f>
@@ -7397,7 +7397,7 @@
         <v>8000</v>
       </c>
       <c r="N63" s="91" t="n">
-        <v>0.3</v>
+        <v>0.3332777731477623</v>
       </c>
       <c r="O63" s="92">
         <f>IF(N63&lt;1, ROUNDUP(M63/(1-N63), -3), M63)</f>
@@ -7496,7 +7496,7 @@
         <v>530000</v>
       </c>
       <c r="N64" s="91" t="n">
-        <v>0.13</v>
+        <v>0.131146116632978</v>
       </c>
       <c r="O64" s="92">
         <f>IF(N64&lt;1, ROUNDUP(M64/(1-N64), -3), M64)</f>
@@ -7605,7 +7605,7 @@
         <v>50000</v>
       </c>
       <c r="N65" s="91" t="n">
-        <v>0.3</v>
+        <v>0.3055459103598661</v>
       </c>
       <c r="O65" s="92">
         <f>IF(N65&lt;1, ROUNDUP(M65/(1-N65), -3), M65)</f>
@@ -7715,7 +7715,7 @@
         <v>169000</v>
       </c>
       <c r="N66" s="91" t="n">
-        <v>0.295833</v>
+        <v>0.2958303992933304</v>
       </c>
       <c r="O66" s="92">
         <f>IF(N66&lt;1, ROUNDUP(M66/(1-N66), -3), M66)</f>
@@ -7828,7 +7828,7 @@
         <v>21700</v>
       </c>
       <c r="N67" s="91" t="n">
-        <v>0.38</v>
+        <v>0.3799822852081488</v>
       </c>
       <c r="O67" s="92">
         <f>IF(N67&lt;1, ROUNDUP(M67/(1-N67), -3), M67)</f>
@@ -7939,7 +7939,7 @@
         <v>45000</v>
       </c>
       <c r="N68" s="91" t="n">
-        <v>0.307692</v>
+        <v>0.3076816566408714</v>
       </c>
       <c r="O68" s="92">
         <f>IF(N68&lt;1, ROUNDUP(M68/(1-N68), -3), M68)</f>
@@ -7989,12 +7989,678 @@
         </is>
       </c>
     </row>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
+    <row r="69">
+      <c r="A69" s="89" t="inlineStr">
+        <is>
+          <t>MTS-0066</t>
+        </is>
+      </c>
+      <c r="B69" s="79" t="inlineStr">
+        <is>
+          <t>Cámara de Seguridad IMOU Ranger 2 Pro 5MP 3K Wi-Fi 360° Smart Tracking</t>
+        </is>
+      </c>
+      <c r="C69" s="80" t="inlineStr">
+        <is>
+          <t>Seguridad y Videovigilancia</t>
+        </is>
+      </c>
+      <c r="D69" s="80" t="inlineStr">
+        <is>
+          <t>IMOU</t>
+        </is>
+      </c>
+      <c r="E69" s="81" t="inlineStr">
+        <is>
+          <t>IPC-S2EN-5R1S-3.6MM</t>
+        </is>
+      </c>
+      <c r="F69" s="81" t="inlineStr">
+        <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G69" s="81" t="inlineStr">
+        <is>
+          <t>6971927236594</t>
+        </is>
+      </c>
+      <c r="H69" s="81" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="I69" s="82" t="inlineStr">
+        <is>
+          <t>🟢 En Stock</t>
+        </is>
+      </c>
+      <c r="J69" s="82" t="n">
+        <v>2</v>
+      </c>
+      <c r="K69" s="81" t="n">
+        <v>2</v>
+      </c>
+      <c r="L69" s="81" t="inlineStr">
+        <is>
+          <t>Vitrina Seguridad / Taller</t>
+        </is>
+      </c>
+      <c r="M69" s="90" t="n">
+        <v>102578</v>
+      </c>
+      <c r="N69" s="91" t="n">
+        <v>0.3507680428357142</v>
+      </c>
+      <c r="O69" s="92">
+        <f>IF(N69&lt;1, ROUNDUP(M69/(1-N69), -3), M69)</f>
+        <v/>
+      </c>
+      <c r="P69" s="91" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="Q69" s="90">
+        <f>IF((1-N69-P69)&gt;0, ROUNDUP((M69+IF(O69&gt;=90000,20000,0))/(1-N69-P69), -3), O69)</f>
+        <v/>
+      </c>
+      <c r="R69" s="90">
+        <f>O69</f>
+        <v/>
+      </c>
+      <c r="S69" s="90">
+        <f>O69-M69</f>
+        <v/>
+      </c>
+      <c r="T69" s="91">
+        <f>IF(O69&gt;0, (O69-M69)/O69, 0)</f>
+        <v/>
+      </c>
+      <c r="U69" s="81" t="inlineStr">
+        <is>
+          <t>12 Meses (1 Año IMOU)</t>
+        </is>
+      </c>
+      <c r="V69" s="80" t="inlineStr">
+        <is>
+          <t>IMAGENES DE PRODUCTOS/camara imou 3K 5MP wifi indoor smart.jpeg</t>
+        </is>
+      </c>
+      <c r="W69" s="80" t="inlineStr">
+        <is>
+          <t>• Resolución: 5 Megapíxeles 3K Ultra HD (2880 x 1620) para máxima nitidez de imagen
+• Cobertura 360°: Giro horizontal de 0~355° e inclinación de -5~80° con seguimiento inteligente de movimiento (Smart Tracking)
+• Visión nocturna avanzada: Infrarrojo claro de hasta 10 metros en oscuridad total
+• Inteligencia Artificial: Detección precisa de humanos y mascotas con alertas instantáneas a la app IMOU Life
+• Audio bidireccional: Micrófono y altavoz integrados para hablar y escuchar en tiempo real
+• Alarma disuasoria: Sirena integrada para ahuyentar intrusos y detección de sonidos anormales
+• Almacenamiento: Ranura para tarjeta Micro SD de hasta 512 GB y opción de almacenamiento en la nube
+• Conectividad: Wi-Fi 2.4 GHz y alimentación moderna por puerto USB Tipo-C.</t>
+        </is>
+      </c>
+      <c r="X69" s="80" t="inlineStr">
+        <is>
+          <t>2 unidades nuevas selladas en taller. Factura FT-18220.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="89" t="inlineStr">
+        <is>
+          <t>MTS-0067</t>
+        </is>
+      </c>
+      <c r="B70" s="79" t="inlineStr">
+        <is>
+          <t>Memoria Micro SD SanDisk Ultra 128GB microSDXC UHS-I Clase 10 (100MB/s)</t>
+        </is>
+      </c>
+      <c r="C70" s="80" t="inlineStr">
+        <is>
+          <t>Almacenamiento y Memorias</t>
+        </is>
+      </c>
+      <c r="D70" s="80" t="inlineStr">
+        <is>
+          <t>SanDisk</t>
+        </is>
+      </c>
+      <c r="E70" s="81" t="inlineStr">
+        <is>
+          <t>SDSQUNR-128G-GN6MN</t>
+        </is>
+      </c>
+      <c r="F70" s="81" t="inlineStr">
+        <is>
+          <t>Rojo / Gris</t>
+        </is>
+      </c>
+      <c r="G70" s="81" t="inlineStr">
+        <is>
+          <t>619659181740</t>
+        </is>
+      </c>
+      <c r="H70" s="81" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="I70" s="82" t="inlineStr">
+        <is>
+          <t>🟢 En Stock</t>
+        </is>
+      </c>
+      <c r="J70" s="82" t="n">
+        <v>3</v>
+      </c>
+      <c r="K70" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="L70" s="81" t="inlineStr">
+        <is>
+          <t>Vitrina Accesorios / Taller</t>
+        </is>
+      </c>
+      <c r="M70" s="90" t="n">
+        <v>90594</v>
+      </c>
+      <c r="N70" s="91" t="n">
+        <v>0.2122192366890147</v>
+      </c>
+      <c r="O70" s="92">
+        <f>IF(N70&lt;1, ROUNDUP(M70/(1-N70), -3), M70)</f>
+        <v/>
+      </c>
+      <c r="P70" s="91" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="Q70" s="90">
+        <f>IF((1-N70-P70)&gt;0, ROUNDUP((M70+IF(O70&gt;=90000,20000,0))/(1-N70-P70), -3), O70)</f>
+        <v/>
+      </c>
+      <c r="R70" s="90">
+        <f>O70</f>
+        <v/>
+      </c>
+      <c r="S70" s="90">
+        <f>O70-M70</f>
+        <v/>
+      </c>
+      <c r="T70" s="91">
+        <f>IF(O70&gt;0, (O70-M70)/O70, 0)</f>
+        <v/>
+      </c>
+      <c r="U70" s="81" t="inlineStr">
+        <is>
+          <t>12 Meses (1 Año SanDisk)</t>
+        </is>
+      </c>
+      <c r="V70" s="80" t="inlineStr">
+        <is>
+          <t>IMAGENES DE PRODUCTOS/micro sd 128gb c10 sandisk.jpeg</t>
+        </is>
+      </c>
+      <c r="W70" s="80" t="inlineStr">
+        <is>
+          <t>• Capacidad: 128 GB de almacenamiento de alta velocidad
+• Velocidad de transferencia: Hasta 100 MB/s de lectura rápida para transferir fotos y videos en segundos
+• Rendimiento: Clase 10, UHS Speed Class 1 (U1) y A1 (optimizada para apps y cámaras)
+• Grabación de video: Optimizada para video Full HD (1080p) continuo y fotografía de alta resolución
+• Resistencia extrema: Diseñada a prueba de agua, golpes, rayos X y temperaturas extremas
+• Compatibilidad: Smartphones, tablets, cámaras de seguridad (IMOU, Tapo, Dahua), drones y Nintendo Switch.</t>
+        </is>
+      </c>
+      <c r="X70" s="80" t="inlineStr">
+        <is>
+          <t>3 unidades nuevas selladas. Pedido Amazon 111-3727652-1457013.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="89" t="inlineStr">
+        <is>
+          <t>MTS-0068</t>
+        </is>
+      </c>
+      <c r="B71" s="79" t="inlineStr">
+        <is>
+          <t>Diadema con Micrófono USB Genius HS-230U para Oficina y Teletrabajo</t>
+        </is>
+      </c>
+      <c r="C71" s="80" t="inlineStr">
+        <is>
+          <t>Periféricos y Accesorios</t>
+        </is>
+      </c>
+      <c r="D71" s="80" t="inlineStr">
+        <is>
+          <t>Genius</t>
+        </is>
+      </c>
+      <c r="E71" s="81" t="inlineStr">
+        <is>
+          <t>HS-230U / 31710021401</t>
+        </is>
+      </c>
+      <c r="F71" s="81" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="G71" s="81" t="inlineStr">
+        <is>
+          <t>4710268257257</t>
+        </is>
+      </c>
+      <c r="H71" s="81" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="I71" s="82" t="inlineStr">
+        <is>
+          <t>🟢 En Stock</t>
+        </is>
+      </c>
+      <c r="J71" s="82" t="n">
+        <v>1</v>
+      </c>
+      <c r="K71" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L71" s="81" t="inlineStr">
+        <is>
+          <t>Vitrina Periféricos / Taller</t>
+        </is>
+      </c>
+      <c r="M71" s="90" t="n">
+        <v>38675</v>
+      </c>
+      <c r="N71" s="91" t="n">
+        <v>0.3554059234320572</v>
+      </c>
+      <c r="O71" s="92">
+        <f>IF(N71&lt;1, ROUNDUP(M71/(1-N71), -3), M71)</f>
+        <v/>
+      </c>
+      <c r="P71" s="91" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="Q71" s="90">
+        <f>IF((1-N71-P71)&gt;0, ROUNDUP((M71+IF(O71&gt;=90000,20000,0))/(1-N71-P71), -3), O71)</f>
+        <v/>
+      </c>
+      <c r="R71" s="90">
+        <f>O71</f>
+        <v/>
+      </c>
+      <c r="S71" s="90">
+        <f>O71-M71</f>
+        <v/>
+      </c>
+      <c r="T71" s="91">
+        <f>IF(O71&gt;0, (O71-M71)/O71, 0)</f>
+        <v/>
+      </c>
+      <c r="U71" s="81" t="inlineStr">
+        <is>
+          <t>12 Meses (1 Año Genius)</t>
+        </is>
+      </c>
+      <c r="V71" s="80" t="inlineStr">
+        <is>
+          <t>IMAGENES DE PRODUCTOS/Diadema usb HS-230U Genius.jpeg</t>
+        </is>
+      </c>
+      <c r="W71" s="80" t="inlineStr">
+        <is>
+          <t>• Conexión: USB Plug &amp; Play inmediata (sin necesidad de controladores ni adaptadores)
+• Micrófono: Micrófono omnidireccional con cancelación de ruido y brazo ajustable y flexible
+• Comodidad: Diadema ultraliviana ajustable con almohadillas acolchadas suaves para largas jornadas
+• Control en cable: Control integrado de volumen y botón de silenciado rápido (Mute)
+• Sonido: Drivers de 30 mm para llamadas nítidas y reproducción clara de audio
+• Compatibilidad: Windows, macOS, Zoom, Microsoft Teams, Google Meet, Skype y teletrabajo.</t>
+        </is>
+      </c>
+      <c r="X71" s="80" t="inlineStr">
+        <is>
+          <t>1 unidad nueva sellada. Factura FT-18220.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="89" t="inlineStr">
+        <is>
+          <t>MTS-0069</t>
+        </is>
+      </c>
+      <c r="B72" s="79" t="inlineStr">
+        <is>
+          <t>Cámara Domo Dahua 2MP Full-Color 1080p Lente 3.6mm Audio Integrado IP67</t>
+        </is>
+      </c>
+      <c r="C72" s="80" t="inlineStr">
+        <is>
+          <t>Seguridad y Videovigilancia</t>
+        </is>
+      </c>
+      <c r="D72" s="80" t="inlineStr">
+        <is>
+          <t>Dahua</t>
+        </is>
+      </c>
+      <c r="E72" s="81" t="inlineStr">
+        <is>
+          <t>DH-HAC-HDW1239TN-A-LED-3.6MM</t>
+        </is>
+      </c>
+      <c r="F72" s="81" t="inlineStr">
+        <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G72" s="81" t="inlineStr">
+        <is>
+          <t>6938596001286</t>
+        </is>
+      </c>
+      <c r="H72" s="81" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="I72" s="82" t="inlineStr">
+        <is>
+          <t>🟢 En Stock</t>
+        </is>
+      </c>
+      <c r="J72" s="82" t="n">
+        <v>2</v>
+      </c>
+      <c r="K72" s="81" t="n">
+        <v>2</v>
+      </c>
+      <c r="L72" s="81" t="inlineStr">
+        <is>
+          <t>Vitrina Seguridad / Taller</t>
+        </is>
+      </c>
+      <c r="M72" s="90" t="n">
+        <v>108528</v>
+      </c>
+      <c r="N72" s="91" t="n">
+        <v>0.3422505590942976</v>
+      </c>
+      <c r="O72" s="92">
+        <f>IF(N72&lt;1, ROUNDUP(M72/(1-N72), -3), M72)</f>
+        <v/>
+      </c>
+      <c r="P72" s="91" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="Q72" s="90">
+        <f>IF((1-N72-P72)&gt;0, ROUNDUP((M72+IF(O72&gt;=90000,20000,0))/(1-N72-P72), -3), O72)</f>
+        <v/>
+      </c>
+      <c r="R72" s="90">
+        <f>O72</f>
+        <v/>
+      </c>
+      <c r="S72" s="90">
+        <f>O72-M72</f>
+        <v/>
+      </c>
+      <c r="T72" s="91">
+        <f>IF(O72&gt;0, (O72-M72)/O72, 0)</f>
+        <v/>
+      </c>
+      <c r="U72" s="81" t="inlineStr">
+        <is>
+          <t>24 Meses (2 Años Dahua)</t>
+        </is>
+      </c>
+      <c r="V72" s="80" t="inlineStr">
+        <is>
+          <t>IMAGENES DE PRODUCTOS/camara ajhua HDCVI 2MP 3.6mm.jpeg</t>
+        </is>
+      </c>
+      <c r="W72" s="80" t="inlineStr">
+        <is>
+          <t>• Tecnología Full-Color 24/7: Imágenes y videos a color las 24 horas del día incluso en oscuridad total
+• Resolución: 2 Megapíxeles 1080p Full HD (1920 x 1080) a 30 fps
+• Lente: Fijo de 3.6 mm con apertura focal F1.6 de alta captación de luz
+• Iluminación LED blanca cálida: Alcance de hasta 20 metros para visión nocturna nítida a color
+• Audio incorporado: Micrófono integrado de alta sensibilidad transmitido por el mismo cable coaxial
+• Formato 4 en 1 conmutable: Compatible con formatos de video CVI, TVI, AHD y CVBS
+• Protección para intemperie: Grado de protección IP67 resistente al agua, lluvia y polvo.</t>
+        </is>
+      </c>
+      <c r="X72" s="80" t="inlineStr">
+        <is>
+          <t>2 unidades nuevas selladas. Factura FT-18220.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="89" t="inlineStr">
+        <is>
+          <t>MTS-0070</t>
+        </is>
+      </c>
+      <c r="B73" s="79" t="inlineStr">
+        <is>
+          <t>Cable Adaptador USB 2.0 a Puerto Serial RS232 DB9 Macho Jaltech</t>
+        </is>
+      </c>
+      <c r="C73" s="80" t="inlineStr">
+        <is>
+          <t>Periféricos y Accesorios</t>
+        </is>
+      </c>
+      <c r="D73" s="80" t="inlineStr">
+        <is>
+          <t>Jaltech</t>
+        </is>
+      </c>
+      <c r="E73" s="81" t="inlineStr">
+        <is>
+          <t>01132 / USB-RS232-DB9</t>
+        </is>
+      </c>
+      <c r="F73" s="81" t="inlineStr">
+        <is>
+          <t>Azul / Negro</t>
+        </is>
+      </c>
+      <c r="G73" s="81" t="inlineStr">
+        <is>
+          <t>Sin código</t>
+        </is>
+      </c>
+      <c r="H73" s="81" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="I73" s="82" t="inlineStr">
+        <is>
+          <t>🟢 En Stock</t>
+        </is>
+      </c>
+      <c r="J73" s="82" t="n">
+        <v>1</v>
+      </c>
+      <c r="K73" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L73" s="81" t="inlineStr">
+        <is>
+          <t>Vitrina Accesorios / Taller</t>
+        </is>
+      </c>
+      <c r="M73" s="90" t="n">
+        <v>14000</v>
+      </c>
+      <c r="N73" s="91" t="n">
+        <v>0.4399775991039642</v>
+      </c>
+      <c r="O73" s="92">
+        <f>IF(N73&lt;1, ROUNDUP(M73/(1-N73), -3), M73)</f>
+        <v/>
+      </c>
+      <c r="P73" s="91" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="Q73" s="90">
+        <f>IF((1-N73-P73)&gt;0, ROUNDUP((M73+IF(O73&gt;=90000,20000,0))/(1-N73-P73), -3), O73)</f>
+        <v/>
+      </c>
+      <c r="R73" s="90">
+        <f>O73</f>
+        <v/>
+      </c>
+      <c r="S73" s="90">
+        <f>O73-M73</f>
+        <v/>
+      </c>
+      <c r="T73" s="91">
+        <f>IF(O73&gt;0, (O73-M73)/O73, 0)</f>
+        <v/>
+      </c>
+      <c r="U73" s="81" t="inlineStr">
+        <is>
+          <t>6 Meses</t>
+        </is>
+      </c>
+      <c r="V73" s="80" t="inlineStr">
+        <is>
+          <t>IMAGENES DE PRODUCTOS/Cable usb a puerto serial RS232.jpeg</t>
+        </is>
+      </c>
+      <c r="W73" s="80" t="inlineStr">
+        <is>
+          <t>• Conector: USB 2.0 Macho a Conector Serial DB9 (RS232) Macho
+• Chipset: Controlador de alta compatibilidad para comunicación serial estable y sin pérdidas
+• Tasa de transferencia: Soporta velocidades de datos de hasta 1 Mbps
+• Aplicaciones: Conexión de impresoras POS/fiscales, balanzas, switches, routers Cisco, PLCs y GPS
+• Compatibilidad: Funciona en Windows 11, 10, 8.1, 7, Linux y macOS.</t>
+        </is>
+      </c>
+      <c r="X73" s="80" t="inlineStr">
+        <is>
+          <t>1 unidad nueva. Cable adaptador USB a serial RS232.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="89" t="inlineStr">
+        <is>
+          <t>MTS-0071</t>
+        </is>
+      </c>
+      <c r="B74" s="79" t="inlineStr">
+        <is>
+          <t>Ventilador Cooler Fan 40x40x10mm 12V 0.1A para DVR, Mini PC e Impresoras 3D</t>
+        </is>
+      </c>
+      <c r="C74" s="80" t="inlineStr">
+        <is>
+          <t>Componentes y Repuestos</t>
+        </is>
+      </c>
+      <c r="D74" s="80" t="inlineStr">
+        <is>
+          <t>Genérico / OEM</t>
+        </is>
+      </c>
+      <c r="E74" s="81" t="inlineStr">
+        <is>
+          <t>FAN-4010-12V</t>
+        </is>
+      </c>
+      <c r="F74" s="81" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="G74" s="81" t="inlineStr">
+        <is>
+          <t>Sin código</t>
+        </is>
+      </c>
+      <c r="H74" s="81" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="I74" s="82" t="inlineStr">
+        <is>
+          <t>🟢 En Stock</t>
+        </is>
+      </c>
+      <c r="J74" s="82" t="n">
+        <v>1</v>
+      </c>
+      <c r="K74" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L74" s="81" t="inlineStr">
+        <is>
+          <t>Taller - Repuestos</t>
+        </is>
+      </c>
+      <c r="M74" s="90" t="n">
+        <v>11000</v>
+      </c>
+      <c r="N74" s="91" t="n">
+        <v>0.4499724986249313</v>
+      </c>
+      <c r="O74" s="92">
+        <f>IF(N74&lt;1, ROUNDUP(M74/(1-N74), -3), M74)</f>
+        <v/>
+      </c>
+      <c r="P74" s="91" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="Q74" s="90">
+        <f>IF((1-N74-P74)&gt;0, ROUNDUP((M74+IF(O74&gt;=90000,20000,0))/(1-N74-P74), -3), O74)</f>
+        <v/>
+      </c>
+      <c r="R74" s="90">
+        <f>O74</f>
+        <v/>
+      </c>
+      <c r="S74" s="90">
+        <f>O74-M74</f>
+        <v/>
+      </c>
+      <c r="T74" s="91">
+        <f>IF(O74&gt;0, (O74-M74)/O74, 0)</f>
+        <v/>
+      </c>
+      <c r="U74" s="81" t="inlineStr">
+        <is>
+          <t>3 Meses</t>
+        </is>
+      </c>
+      <c r="V74" s="80" t="inlineStr">
+        <is>
+          <t>IMAGENES DE PRODUCTOS/Ventilador para dvr .jpeg</t>
+        </is>
+      </c>
+      <c r="W74" s="80" t="inlineStr">
+        <is>
+          <t>• Dimensiones: 40 mm x 40 mm x 10 mm (1.5 pulgadas aprox.)
+• Alimentación: 12V DC a 0.1 Amperios (bajo consumo y operación silenciosa)
+• Conector: Terminal estándar de 2 pines (rojo positivo / negro negativo)
+• Aplicaciones: Extractor de calor y disipador de reemplazo para grabadores DVR/NVR (Dahua, Hikvision), mini PCs, impresoras 3D, routers y fuentes de poder.</t>
+        </is>
+      </c>
+      <c r="X74" s="80" t="inlineStr">
+        <is>
+          <t>1 unidad nueva. Ventilador micro cooler 4010 12V 0.1A.</t>
+        </is>
+      </c>
+    </row>
     <row r="75"/>
     <row r="76"/>
     <row r="77"/>

</xml_diff>

<commit_message>
Actualización desde Panel Admin Local
</commit_message>
<xml_diff>
--- a/inventario_max_technology_store.xlsx
+++ b/inventario_max_technology_store.xlsx
@@ -8050,7 +8050,7 @@
         <v>102578</v>
       </c>
       <c r="N69" s="91" t="n">
-        <v>0.3507680428357142</v>
+        <v>0.265</v>
       </c>
       <c r="O69" s="92">
         <f>IF(N69&lt;1, ROUNDUP(M69/(1-N69), -3), M69)</f>
@@ -8276,7 +8276,7 @@
         <v>38675</v>
       </c>
       <c r="N71" s="91" t="n">
-        <v>0.3554059234320572</v>
+        <v>0.14</v>
       </c>
       <c r="O71" s="92">
         <f>IF(N71&lt;1, ROUNDUP(M71/(1-N71), -3), M71)</f>
@@ -8388,7 +8388,7 @@
         <v>108528</v>
       </c>
       <c r="N72" s="91" t="n">
-        <v>0.3422505590942976</v>
+        <v>0.2</v>
       </c>
       <c r="O72" s="92">
         <f>IF(N72&lt;1, ROUNDUP(M72/(1-N72), -3), M72)</f>
@@ -8501,7 +8501,7 @@
         <v>14000</v>
       </c>
       <c r="N73" s="91" t="n">
-        <v>0.4399775991039642</v>
+        <v>0.3</v>
       </c>
       <c r="O73" s="92">
         <f>IF(N73&lt;1, ROUNDUP(M73/(1-N73), -3), M73)</f>
@@ -8612,7 +8612,7 @@
         <v>11000</v>
       </c>
       <c r="N74" s="91" t="n">
-        <v>0.4499724986249313</v>
+        <v>0.22</v>
       </c>
       <c r="O74" s="92">
         <f>IF(N74&lt;1, ROUNDUP(M74/(1-N74), -3), M74)</f>

</xml_diff>

<commit_message>
Ingreso de nuevas compras (Facturas FT-20168, FT-20171, FT-20172 y FEVO-34572): Nuevos productos MTS-0073 a MTS-0076 y actualizacion de stock en MTS-0033, MTS-0037 y MTS-0061
</commit_message>
<xml_diff>
--- a/inventario_max_technology_store.xlsx
+++ b/inventario_max_technology_store.xlsx
@@ -4614,11 +4614,11 @@
       </c>
       <c r="I36" s="72" t="inlineStr">
         <is>
-          <t>⚪ Agotado</t>
+          <t>🟢 En Stock</t>
         </is>
       </c>
       <c r="J36" s="73" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K36" s="74" t="n">
         <v>10</v>
@@ -4629,10 +4629,10 @@
         </is>
       </c>
       <c r="M36" s="75" t="n">
-        <v>158550</v>
+        <v>152338</v>
       </c>
       <c r="N36" s="76" t="n">
-        <v>0.2825759392576437</v>
+        <v>0.31068466373151</v>
       </c>
       <c r="O36" s="77">
         <f>IF(N36&lt;1, ROUNDUP(M36/(1-N36), -3), M36)</f>
@@ -4674,7 +4674,7 @@
       </c>
       <c r="X36" s="69" t="inlineStr">
         <is>
-          <t>Producto de alta rotación para oficinas y hogares.</t>
+          <t>Producto de alta rotación para oficinas y hogares. | 3 unidades nuevas ingresadas (Factura FT-20168).</t>
         </is>
       </c>
     </row>
@@ -5030,11 +5030,11 @@
       </c>
       <c r="I40" s="72" t="inlineStr">
         <is>
-          <t>⚪ Agotado</t>
+          <t>🟢 En Stock</t>
         </is>
       </c>
       <c r="J40" s="73" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K40" s="74" t="n">
         <v>11</v>
@@ -5045,10 +5045,10 @@
         </is>
       </c>
       <c r="M40" s="75" t="n">
-        <v>311071</v>
+        <v>316143</v>
       </c>
       <c r="N40" s="76" t="n">
-        <v>0.2023800061025798</v>
+        <v>0.1893748445508835</v>
       </c>
       <c r="O40" s="77">
         <f>IF(N40&lt;1, ROUNDUP(M40/(1-N40), -3), M40)</f>
@@ -5096,7 +5096,7 @@
       </c>
       <c r="X40" s="69" t="inlineStr">
         <is>
-          <t>10 unidades físicas selladas. Seriales: BLR01916302500002 a BLR01916302500646. Factura FT-9364.</t>
+          <t>10 unidades físicas selladas. Seriales: BLR01916302500002 a BLR01916302500646. Factura FT-9364. | 3 unidades nuevas ingresadas (Factura FT-20171).</t>
         </is>
       </c>
     </row>
@@ -7482,10 +7482,10 @@
         </is>
       </c>
       <c r="J64" s="82" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K64" s="81" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L64" s="81" t="inlineStr">
         <is>
@@ -7542,7 +7542,11 @@
 • Compatible con PCs de escritorio y portátiles con slot M.2 NVMe.</t>
         </is>
       </c>
-      <c r="X64" s="80" t="inlineStr"/>
+      <c r="X64" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | 1 unidad nueva ingresada (Serial: 4P2220399418, Factura FEVO 34572).</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="89" t="inlineStr">
@@ -8887,10 +8891,457 @@
       </c>
       <c r="X76" s="80" t="inlineStr"/>
     </row>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
+    <row r="77">
+      <c r="A77" s="89" t="inlineStr">
+        <is>
+          <t>MTS-0073</t>
+        </is>
+      </c>
+      <c r="B77" s="79" t="inlineStr">
+        <is>
+          <t>Cámara de Seguridad IMOU Ranger 2 Dual 10MP (5MP+5MP) Wi-Fi 6 360° Smart Full-Color</t>
+        </is>
+      </c>
+      <c r="C77" s="80" t="inlineStr">
+        <is>
+          <t>Seguridad y Videovigilancia</t>
+        </is>
+      </c>
+      <c r="D77" s="80" t="inlineStr">
+        <is>
+          <t>IMOU</t>
+        </is>
+      </c>
+      <c r="E77" s="81" t="inlineStr">
+        <is>
+          <t>IPC-S20EN-10M0S-3.6MM</t>
+        </is>
+      </c>
+      <c r="F77" s="81" t="inlineStr">
+        <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G77" s="81" t="inlineStr">
+        <is>
+          <t>Sin código</t>
+        </is>
+      </c>
+      <c r="H77" s="81" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="I77" s="82" t="inlineStr">
+        <is>
+          <t>🟢 En Stock</t>
+        </is>
+      </c>
+      <c r="J77" s="82" t="n">
+        <v>2</v>
+      </c>
+      <c r="K77" s="81" t="n">
+        <v>2</v>
+      </c>
+      <c r="L77" s="81" t="inlineStr">
+        <is>
+          <t>Vitrina Seguridad / Taller</t>
+        </is>
+      </c>
+      <c r="M77" s="90" t="n">
+        <v>187400</v>
+      </c>
+      <c r="N77" s="91" t="n">
+        <v>0.3007436594912668</v>
+      </c>
+      <c r="O77" s="92">
+        <f>IF(N77&lt;1, ROUNDUP(M77/(1-N77), -3), M77)</f>
+        <v/>
+      </c>
+      <c r="P77" s="91" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="Q77" s="90">
+        <f>IF((1-N77-P77)&gt;0, ROUNDUP((M77+IF(O77&gt;=90000,20000,0))/(1-N77-P77), -3), O77)</f>
+        <v/>
+      </c>
+      <c r="R77" s="90">
+        <f>O77</f>
+        <v/>
+      </c>
+      <c r="S77" s="90">
+        <f>O77-M77</f>
+        <v/>
+      </c>
+      <c r="T77" s="91">
+        <f>IF(O77&gt;0, (O77-M77)/O77, 0)</f>
+        <v/>
+      </c>
+      <c r="U77" s="81" t="inlineStr">
+        <is>
+          <t>12 Meses (1 Año Oficial IMOU)</t>
+        </is>
+      </c>
+      <c r="V77" s="80" t="inlineStr">
+        <is>
+          <t>identidad visual max tech/Logo MAX Tech.png</t>
+        </is>
+      </c>
+      <c r="W77" s="80" t="inlineStr">
+        <is>
+          <t>• Doble lente de 10MP en total: Lente fijo 5MP 3K + Lente robótico PT 5MP 3K con giro 360° e inclinación
+• Cobertura simultánea: Monitorea dos áreas al mismo tiempo con una sola cámara
+• Visión nocturna Smart Full-Color: 4 modos inteligentes de visión nocturna a todo color
+• Conectividad Wi-Fi 6 (2.4 GHz y 5 GHz) de alta velocidad y máxima estabilidad de señal
+• Detección inteligente por IA: Reconoce humanos y mascotas con seguimiento automático de movimiento
+• Audio bidireccional y botón de llamada directa (One-touch call) desde la cámara al celular
+• Sirena y alarma disuasoria con detección de sonidos anormales
+• Puerto de alimentación USB-C y ranura para tarjeta Micro SD de hasta 512 GB.</t>
+        </is>
+      </c>
+      <c r="X77" s="80" t="inlineStr">
+        <is>
+          <t>2 unidades nuevas selladas en taller. Factura FT-20168.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="89" t="inlineStr">
+        <is>
+          <t>MTS-0074</t>
+        </is>
+      </c>
+      <c r="B78" s="79" t="inlineStr">
+        <is>
+          <t>Router TP-Link Archer BE550 Tribanda Wi-Fi 7 BE9300 9.3Gbps Puertos 2.5G</t>
+        </is>
+      </c>
+      <c r="C78" s="80" t="inlineStr">
+        <is>
+          <t>Redes y Conectividad</t>
+        </is>
+      </c>
+      <c r="D78" s="80" t="inlineStr">
+        <is>
+          <t>TP-Link</t>
+        </is>
+      </c>
+      <c r="E78" s="81" t="inlineStr">
+        <is>
+          <t>Archer BE550</t>
+        </is>
+      </c>
+      <c r="F78" s="81" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="G78" s="81" t="inlineStr">
+        <is>
+          <t>Sin código</t>
+        </is>
+      </c>
+      <c r="H78" s="81" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="I78" s="82" t="inlineStr">
+        <is>
+          <t>🟢 En Stock</t>
+        </is>
+      </c>
+      <c r="J78" s="82" t="n">
+        <v>1</v>
+      </c>
+      <c r="K78" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L78" s="81" t="inlineStr">
+        <is>
+          <t>Estante Redes / Taller</t>
+        </is>
+      </c>
+      <c r="M78" s="90" t="n">
+        <v>798490</v>
+      </c>
+      <c r="N78" s="91" t="n">
+        <v>0.2007099106205311</v>
+      </c>
+      <c r="O78" s="92">
+        <f>IF(N78&lt;1, ROUNDUP(M78/(1-N78), -3), M78)</f>
+        <v/>
+      </c>
+      <c r="P78" s="91" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="Q78" s="90">
+        <f>IF((1-N78-P78)&gt;0, ROUNDUP((M78+IF(O78&gt;=90000,20000,0))/(1-N78-P78), -3), O78)</f>
+        <v/>
+      </c>
+      <c r="R78" s="90">
+        <f>O78</f>
+        <v/>
+      </c>
+      <c r="S78" s="90">
+        <f>O78-M78</f>
+        <v/>
+      </c>
+      <c r="T78" s="91">
+        <f>IF(O78&gt;0, (O78-M78)/O78, 0)</f>
+        <v/>
+      </c>
+      <c r="U78" s="81" t="inlineStr">
+        <is>
+          <t>24 Meses (2 Años Oficial TP-Link)</t>
+        </is>
+      </c>
+      <c r="V78" s="80" t="inlineStr">
+        <is>
+          <t>identidad visual max tech/Logo MAX Tech.png</t>
+        </is>
+      </c>
+      <c r="W78" s="80" t="inlineStr">
+        <is>
+          <t>• Tecnología Wi-Fi 7 de última generación con velocidad tribanda extrema de hasta 9.300 Mbps (9.3 Gbps)
+• Operación Multi-Link (MLO) y canales de 320 MHz para latencia ultrabaja y máxima estabilidad
+• 5 puertos Ethernet 2.5 Gbps (1 puerto WAN 2.5G + 4 puertos LAN 2.5G) ideales para fibra óptica ultrarrápida
+• 6 antenas internas óptimamente posicionadas con tecnología Beamforming para cobertura omnidireccional
+• Puerto USB 3.0 de alta velocidad para compartir archivos y crear almacenamiento NAS local
+• Procesador de alta potencia para streaming 8K/4K simultáneo, gaming profesional y realidad virtual (VR)
+• Seguridad avanzada TP-Link HomeShield y compatibilidad con EasyMesh.</t>
+        </is>
+      </c>
+      <c r="X78" s="80" t="inlineStr">
+        <is>
+          <t>1 unidad nueva sellada. Factura FT-20172.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="89" t="inlineStr">
+        <is>
+          <t>MTS-0075</t>
+        </is>
+      </c>
+      <c r="B79" s="79" t="inlineStr">
+        <is>
+          <t>Disco Estado Sólido SSD 2.5" SATA III 1TB (1000GB) ADATA Ultimate SU650</t>
+        </is>
+      </c>
+      <c r="C79" s="80" t="inlineStr">
+        <is>
+          <t>Almacenamiento y Memorias</t>
+        </is>
+      </c>
+      <c r="D79" s="80" t="inlineStr">
+        <is>
+          <t>ADATA</t>
+        </is>
+      </c>
+      <c r="E79" s="81" t="inlineStr">
+        <is>
+          <t>ASU650SS-1TT-R / SU650 1TB</t>
+        </is>
+      </c>
+      <c r="F79" s="81" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="G79" s="81" t="inlineStr">
+        <is>
+          <t>Sin código</t>
+        </is>
+      </c>
+      <c r="H79" s="81" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="I79" s="82" t="inlineStr">
+        <is>
+          <t>🟢 En Stock</t>
+        </is>
+      </c>
+      <c r="J79" s="82" t="n">
+        <v>1</v>
+      </c>
+      <c r="K79" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L79" s="81" t="inlineStr">
+        <is>
+          <t>Vitrina Accesorios / Taller</t>
+        </is>
+      </c>
+      <c r="M79" s="90" t="n">
+        <v>515000</v>
+      </c>
+      <c r="N79" s="91" t="n">
+        <v>0.2015491496886042</v>
+      </c>
+      <c r="O79" s="92">
+        <f>IF(N79&lt;1, ROUNDUP(M79/(1-N79), -3), M79)</f>
+        <v/>
+      </c>
+      <c r="P79" s="91" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="Q79" s="90">
+        <f>IF((1-N79-P79)&gt;0, ROUNDUP((M79+IF(O79&gt;=90000,20000,0))/(1-N79-P79), -3), O79)</f>
+        <v/>
+      </c>
+      <c r="R79" s="90">
+        <f>O79</f>
+        <v/>
+      </c>
+      <c r="S79" s="90">
+        <f>O79-M79</f>
+        <v/>
+      </c>
+      <c r="T79" s="91">
+        <f>IF(O79&gt;0, (O79-M79)/O79, 0)</f>
+        <v/>
+      </c>
+      <c r="U79" s="81" t="inlineStr">
+        <is>
+          <t>36 Meses (3 Años Oficial ADATA)</t>
+        </is>
+      </c>
+      <c r="V79" s="80" t="inlineStr">
+        <is>
+          <t>identidad visual max tech/Logo MAX Tech.png</t>
+        </is>
+      </c>
+      <c r="W79" s="80" t="inlineStr">
+        <is>
+          <t>• Capacidad: 1 TB (1.000 GB) de almacenamiento sólido
+• Factor de forma: 2.5 pulgadas (7 mm de grosor, ultrafino)
+• Interfaz: SATA III 6Gb/s (retrocompatible con SATA II)
+• Velocidad de lectura secuencial: Hasta 520 MB/s
+• Velocidad de escritura secuencial: Hasta 450 MB/s
+• Tecnología: Memoria 3D NAND Flash con caché SLC y corrección de errores ECC
+• Ideal para repotenciar portátiles y computadores de escritorio con máxima capacidad y velocidad.</t>
+        </is>
+      </c>
+      <c r="X79" s="80" t="inlineStr">
+        <is>
+          <t>1 unidad nueva sellada. Serial: 4P3621895537. Factura FEVO 34572.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="89" t="inlineStr">
+        <is>
+          <t>MTS-0076</t>
+        </is>
+      </c>
+      <c r="B80" s="79" t="inlineStr">
+        <is>
+          <t>Caja / Cofre Externo para Disco SSD M.2 NVMe a USB 3.0 / USB-C Negro</t>
+        </is>
+      </c>
+      <c r="C80" s="80" t="inlineStr">
+        <is>
+          <t>Almacenamiento y Memorias</t>
+        </is>
+      </c>
+      <c r="D80" s="80" t="inlineStr">
+        <is>
+          <t>Digital MTX / OEM</t>
+        </is>
+      </c>
+      <c r="E80" s="81" t="inlineStr">
+        <is>
+          <t>00003583 / CASE-M2-NVME-USB</t>
+        </is>
+      </c>
+      <c r="F80" s="81" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="G80" s="81" t="inlineStr">
+        <is>
+          <t>Sin código</t>
+        </is>
+      </c>
+      <c r="H80" s="81" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="I80" s="82" t="inlineStr">
+        <is>
+          <t>🟢 En Stock</t>
+        </is>
+      </c>
+      <c r="J80" s="82" t="n">
+        <v>1</v>
+      </c>
+      <c r="K80" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L80" s="81" t="inlineStr">
+        <is>
+          <t>Vitrina Accesorios / Taller</t>
+        </is>
+      </c>
+      <c r="M80" s="90" t="n">
+        <v>45000</v>
+      </c>
+      <c r="N80" s="91" t="n">
+        <v>0.3382255621406197</v>
+      </c>
+      <c r="O80" s="92">
+        <f>IF(N80&lt;1, ROUNDUP(M80/(1-N80), -3), M80)</f>
+        <v/>
+      </c>
+      <c r="P80" s="91" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="Q80" s="90">
+        <f>IF((1-N80-P80)&gt;0, ROUNDUP((M80+IF(O80&gt;=90000,20000,0))/(1-N80-P80), -3), O80)</f>
+        <v/>
+      </c>
+      <c r="R80" s="90">
+        <f>O80</f>
+        <v/>
+      </c>
+      <c r="S80" s="90">
+        <f>O80-M80</f>
+        <v/>
+      </c>
+      <c r="T80" s="91">
+        <f>IF(O80&gt;0, (O80-M80)/O80, 0)</f>
+        <v/>
+      </c>
+      <c r="U80" s="81" t="inlineStr">
+        <is>
+          <t>3 Meses</t>
+        </is>
+      </c>
+      <c r="V80" s="80" t="inlineStr">
+        <is>
+          <t>identidad visual max tech/Logo MAX Tech.png</t>
+        </is>
+      </c>
+      <c r="W80" s="80" t="inlineStr">
+        <is>
+          <t>• Compatibilidad: Discos sólidos SSD M.2 NVMe PCIe M-Key y B+M Key (tamaños 2230, 2242, 2260, 2280)
+• Conexión: Interfaz USB 3.0 / USB-C de alta velocidad (transferencias de hasta 10 Gbps)
+• Carcasa: Construcción metálica en aluminio negro para disipación térmica óptima
+• Instalación fácil y rápida sin herramientas complicadas
+• Plug &amp; Play: Compatible con Windows, macOS, Linux, Smart TV y consolas de videojuegos.</t>
+        </is>
+      </c>
+      <c r="X80" s="80" t="inlineStr">
+        <is>
+          <t>1 unidad nueva. Factura FEVO 34572.</t>
+        </is>
+      </c>
+    </row>
     <row r="81"/>
     <row r="82"/>
     <row r="83"/>

</xml_diff>

<commit_message>
Asignacion de fotografias a productos MTS-0033 (UPS Unipower), MTS-0073 (IMOU Ranger 2 Dual), MTS-0075 (SSD ADATA SU650 1TB) y MTS-0076 (Caja M.2 NVMe USB)
</commit_message>
<xml_diff>
--- a/inventario_max_technology_store.xlsx
+++ b/inventario_max_technology_store.xlsx
@@ -4664,7 +4664,7 @@
       </c>
       <c r="V36" s="69" t="inlineStr">
         <is>
-          <t>identidad visual max tech/Logo MAX Tech.png</t>
+          <t>IMAGENES DE PRODUCTOS/ups unipower.jpg</t>
         </is>
       </c>
       <c r="W36" s="69" t="inlineStr">
@@ -8984,7 +8984,7 @@
       </c>
       <c r="V77" s="80" t="inlineStr">
         <is>
-          <t>identidad visual max tech/Logo MAX Tech.png</t>
+          <t>IMAGENES DE PRODUCTOS/IMOU CAMARA DUAL.jpg</t>
         </is>
       </c>
       <c r="W77" s="80" t="inlineStr">
@@ -9211,7 +9211,7 @@
       </c>
       <c r="V79" s="80" t="inlineStr">
         <is>
-          <t>identidad visual max tech/Logo MAX Tech.png</t>
+          <t>IMAGENES DE PRODUCTOS/Disco SSD 2.5 ADATA SU650 de 1TB.jpg</t>
         </is>
       </c>
       <c r="W79" s="80" t="inlineStr">
@@ -9324,7 +9324,7 @@
       </c>
       <c r="V80" s="80" t="inlineStr">
         <is>
-          <t>identidad visual max tech/Logo MAX Tech.png</t>
+          <t>IMAGENES DE PRODUCTOS/Caja-DiscoDuro-NVME-USB3-7326-1.webp</t>
         </is>
       </c>
       <c r="W80" s="80" t="inlineStr">

</xml_diff>